<commit_message>
feat: auto sync with Google Apps Script web app endpoint (表單回覆1 tab) with local fallback
</commit_message>
<xml_diff>
--- a/reports_excel/主管專用_【何維安】部屬自評vs主管評對照表.xlsx
+++ b/reports_excel/主管專用_【何維安】部屬自評vs主管評對照表.xlsx
@@ -892,7 +892,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="34" customHeight="1">
+    <row r="15" ht="24" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>其他創造的好事與預防的壞事</t>
@@ -905,7 +905,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>想要和大家一起創造Work Life Balance，並且避免大家有超出自己職務與專業範圍的工作產生。</t>
+          <t>（部屬未填寫自評實例）</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">

</xml_diff>